<commit_message>
Development of Data Import Module
Added LD Advance Adjustment option in invoice sample sheet
</commit_message>
<xml_diff>
--- a/app/assets/data-import-samples/invoice/invoice.xlsx
+++ b/app/assets/data-import-samples/invoice/invoice.xlsx
@@ -140,9 +140,6 @@
     <t>(Only No)</t>
   </si>
   <si>
-    <t>(Material Advance/Interest Recovery/Mob Advance Adjustment/Erection Advance/Other Deductions)</t>
-  </si>
-  <si>
     <t>Credit Invoice Amount</t>
   </si>
   <si>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>ORG ID</t>
+  </si>
+  <si>
+    <t>(Material Advance/Interest Recovery/Mob Advance Adjustment/Erection Advance/LD Advance Adjustment/Other Deductions)</t>
   </si>
 </sst>
 </file>
@@ -555,7 +555,7 @@
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -579,7 +579,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -666,16 +666,16 @@
         <v>35</v>
       </c>
       <c r="AL1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
@@ -729,7 +729,7 @@
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
       <c r="AJ2" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="AK2" s="2"/>
       <c r="AL2" s="2"/>

</xml_diff>